<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 21:47 UTC
</commit_message>
<xml_diff>
--- a/data/50001500 - EQ MIN LA HACIENDA.xlsx
+++ b/data/50001500 - EQ MIN LA HACIENDA.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="275">
   <si>
     <t xml:space="preserve">50001500 - EQ .MIN  LA HACIENDA </t>
   </si>
@@ -187,622 +187,622 @@
     <t>Ingenieria Servicios:,Coordinacion Entrega con Cliente</t>
   </si>
   <si>
+    <t>1214061368086214</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4214 - TABLERO DE FUERZA SS </t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>1213247778168598</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria basica Rodete,Ingenieria Basica Motor,Analisis de costeo</t>
+  </si>
+  <si>
+    <t>1213247778168600</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+  </si>
+  <si>
+    <t>1213247778168601</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta Nucleo rodete,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213247778168602</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Planos Preliminar</t>
+  </si>
+  <si>
+    <t>1213247778168603</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
+    <t>1213247778168604</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta motor,propuesta tableros,propuesta Nucleo rodete,propuesta alabes,propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213247778168605</t>
+  </si>
+  <si>
+    <t>propuesta motor</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC motor</t>
+  </si>
+  <si>
+    <t>1213247778168606</t>
+  </si>
+  <si>
+    <t>propuesta alabes</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Alabe</t>
+  </si>
+  <si>
+    <t>1213247778168607</t>
+  </si>
+  <si>
+    <t>propuesta tableros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4214 </t>
+  </si>
+  <si>
+    <t>1213247778168608</t>
+  </si>
+  <si>
+    <t>propuesta Nucleo rodete</t>
+  </si>
+  <si>
+    <t>benjamin.bustos@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>1213247778168609</t>
+  </si>
+  <si>
+    <t>propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>hugo isla martinez</t>
+  </si>
+  <si>
+    <t>hugo.isla@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC materiales</t>
+  </si>
+  <si>
+    <t>1213247778168610</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Alabe,Tableros OT 4214 ,rodete,Motor,Materiales a codigo // compras locales aprovisionamientomiento</t>
+  </si>
+  <si>
+    <t>1213247778168611</t>
+  </si>
+  <si>
+    <t>Alabe</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe,Fabricación Alabe</t>
+  </si>
+  <si>
+    <t>1213247781640415</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe,Alabe</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
+  </si>
+  <si>
+    <t>1213247781640416</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe</t>
+  </si>
+  <si>
+    <t>Alabe,Recepcion Alabe,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1213247781640417</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableros OT 4214 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Tableros OT 4214 ,Fabricación Tablero OT 4214 </t>
+  </si>
+  <si>
+    <t>1213247781640418</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Tableros OT 4214 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Tablero OT 4214 ,Tableros OT 4214 </t>
+  </si>
+  <si>
+    <t>1213247781640419</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Tablero OT 4214 </t>
+  </si>
+  <si>
+    <t>Tableros OT 4214 ,RecepcionTableros,Recepcion Tableros</t>
+  </si>
+  <si>
+    <t>1213247781640420</t>
+  </si>
+  <si>
+    <t>rodete</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete,Fabricación  Rodete</t>
+  </si>
+  <si>
+    <t>1213247781640421</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>Fabricación  Rodete,rodete</t>
+  </si>
+  <si>
+    <t>1213247781640422</t>
+  </si>
+  <si>
+    <t>Fabricación  Rodete</t>
+  </si>
+  <si>
+    <t>rodete,Recepcion Rodete,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1213247781640423</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>Generación OC motor,Fabricaciónx motor,Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>1213247781640424</t>
+  </si>
+  <si>
+    <t>Generación OC motor</t>
+  </si>
+  <si>
+    <t>Fabricaciónx motor,Motor,Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>1213247781640425</t>
+  </si>
+  <si>
+    <t>Fabricaciónx motor</t>
+  </si>
+  <si>
+    <t>Motor,Recepcion Motor,Recepcion Motor</t>
+  </si>
+  <si>
+    <t>1213247781640426</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>Motor,Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213247781640427</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>1213247781640428</t>
+  </si>
+  <si>
+    <t>Generación OC materiales</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales,Materiales a codigo // compras locales aprovisionamientomiento</t>
+  </si>
+  <si>
+    <t>1213247781640429</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213575386156573</t>
+  </si>
+  <si>
+    <t>Ingenieria Y diseño</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos Definitivos,Check Planos,Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213575386156575</t>
+  </si>
+  <si>
+    <t>Planos Preliminar</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t>Planos Definitivos</t>
+  </si>
+  <si>
+    <t>1213575386156577</t>
+  </si>
+  <si>
+    <t>Planos Preliminar,Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>Check Planos,Ingenieria Y diseño</t>
+  </si>
+  <si>
+    <t>1213575386156579</t>
+  </si>
+  <si>
+    <t>Check Planos</t>
+  </si>
+  <si>
+    <t>Preparación de materiales,Armado,Montaje motor,Montaje Rodete,Montaje Alabe,Ingenieria Y diseño</t>
+  </si>
+  <si>
+    <t>1213575386156581</t>
+  </si>
+  <si>
+    <t>Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t>Pruebas FAT</t>
+  </si>
+  <si>
+    <t>Ingenieria Y diseño,RE-PINTADO</t>
+  </si>
+  <si>
+    <t>1213247781640432</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213247781640433</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
+  </si>
+  <si>
+    <t>1213247781640434</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>Bodega:,Preparación Materiales,Preparación de materiales</t>
+  </si>
+  <si>
+    <t>1213575386156541</t>
+  </si>
+  <si>
+    <t>Caldereria</t>
+  </si>
+  <si>
+    <t>Armado,Preparación de materiales,Control de calidad Aramado</t>
+  </si>
+  <si>
+    <t>1213575386156543</t>
+  </si>
+  <si>
+    <t>Preparación de materiales</t>
+  </si>
+  <si>
+    <t>Nicolás Mol</t>
+  </si>
+  <si>
+    <t>nicolas.mol@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Check Planos</t>
+  </si>
+  <si>
+    <t>1213575386156545</t>
+  </si>
+  <si>
+    <t>Armado</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,Check Planos</t>
+  </si>
+  <si>
+    <t>Control de calidad Aramado,Caldereria</t>
+  </si>
+  <si>
+    <t>1213575386156547</t>
+  </si>
+  <si>
+    <t>Control de calidad Aramado</t>
+  </si>
+  <si>
+    <t>Caldereria,Revestimiento</t>
+  </si>
+  <si>
+    <t>1213575386156613</t>
+  </si>
+  <si>
+    <t>bodega</t>
+  </si>
+  <si>
+    <t>Recepcion Motor,Recepcion Rodete,Recepcion Tableros,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1213575386156621</t>
+  </si>
+  <si>
+    <t>Recepcion Motor</t>
+  </si>
+  <si>
+    <t>bodega,Montaje motor</t>
+  </si>
+  <si>
+    <t>1213575386156619</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>bodega,Montaje Rodete</t>
+  </si>
+  <si>
+    <t>1213575386156617</t>
+  </si>
+  <si>
+    <t>bodega,Revision tableros pruebas</t>
+  </si>
+  <si>
+    <t>1213575386156615</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>bodega,Montaje Alabe</t>
+  </si>
+  <si>
+    <t>1213247781640444</t>
+  </si>
+  <si>
+    <t>Montaje:</t>
+  </si>
+  <si>
+    <t>Revestimiento,Montaje motor,Montaje Rodete,Montaje Alabe,Pruebas FAT,RE-PINTADO</t>
+  </si>
+  <si>
+    <t>1213247781640445</t>
+  </si>
+  <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>Montaje motor,Montaje Rodete,Montaje Alabe,Montaje:,Montaje motor</t>
+  </si>
+  <si>
+    <t>1213247781640446</t>
+  </si>
+  <si>
+    <t>Montaje motor</t>
+  </si>
+  <si>
+    <t>Revestimiento,Check Planos,Recepcion Motor</t>
+  </si>
+  <si>
+    <t>Pruebas FAT,Montaje:</t>
+  </si>
+  <si>
+    <t>1213247781640448</t>
+  </si>
+  <si>
+    <t>Montaje Rodete</t>
+  </si>
+  <si>
+    <t>Revestimiento,Check Planos,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1213247781640447</t>
+  </si>
+  <si>
+    <t>Montaje Alabe</t>
+  </si>
+  <si>
+    <t>Revestimiento,Check Planos,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1213247781640449</t>
+  </si>
+  <si>
+    <t>Montaje motor,Montaje Rodete,Montaje Alabe</t>
+  </si>
+  <si>
+    <t>Montaje:,Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213247781640450</t>
+  </si>
+  <si>
+    <t>RE-PINTADO</t>
+  </si>
+  <si>
+    <t>Montaje:,Coordinacion Entrega con Cliente</t>
+  </si>
+  <si>
+    <t>1213247781640451</t>
+  </si>
+  <si>
+    <t>Logistica:</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
+  </si>
+  <si>
+    <t>1213247781640452</t>
+  </si>
+  <si>
+    <t>Karin Pinto</t>
+  </si>
+  <si>
+    <t>kpinto@zitron.com</t>
+  </si>
+  <si>
+    <t>RE-PINTADO,OT 4214 - TABLERO DE FUERZA SS ,Revision tableros pruebas</t>
+  </si>
+  <si>
+    <t>Logistica:,Embalaje</t>
+  </si>
+  <si>
+    <t>1213247781640453</t>
+  </si>
+  <si>
+    <t>Embalaje</t>
+  </si>
+  <si>
+    <t>PACKING LIST,Logistica:</t>
+  </si>
+  <si>
+    <t>1213247781640454</t>
+  </si>
+  <si>
+    <t>PACKING LIST</t>
+  </si>
+  <si>
+    <t>Despacho,Logistica:</t>
+  </si>
+  <si>
+    <t>1213247781640455</t>
+  </si>
+  <si>
+    <t>Despacho</t>
+  </si>
+  <si>
+    <t>Gestion,Costos,Logistica:,Instalación componentes</t>
+  </si>
+  <si>
+    <t>1213247781640456</t>
+  </si>
+  <si>
+    <t>Cierre proyecto:</t>
+  </si>
+  <si>
+    <t>Gestion,Costos</t>
+  </si>
+  <si>
+    <t>1213247781640457</t>
+  </si>
+  <si>
+    <t>Gestion</t>
+  </si>
+  <si>
+    <t>Nicolás</t>
+  </si>
+  <si>
+    <t>nicolas.tello@zitron.com</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1214061368086214</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4214 - TABLERO DE FUERZA SS </t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente</t>
-  </si>
-  <si>
-    <t>1213247778168598</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria basica Rodete,Ingenieria Basica Motor,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213247778168600</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
-  </si>
-  <si>
-    <t>1213247778168601</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta Nucleo rodete,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213247778168602</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Planos Preliminar</t>
-  </si>
-  <si>
-    <t>1213247778168603</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>1213247778168604</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta motor,propuesta tableros,propuesta Nucleo rodete,propuesta alabes,propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213247778168605</t>
-  </si>
-  <si>
-    <t>propuesta motor</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC motor</t>
-  </si>
-  <si>
-    <t>1213247778168606</t>
-  </si>
-  <si>
-    <t>propuesta alabes</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Alabe</t>
-  </si>
-  <si>
-    <t>1213247778168607</t>
-  </si>
-  <si>
-    <t>propuesta tableros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta compras:,Generación OC Tableros OT 4214 </t>
-  </si>
-  <si>
-    <t>1213247778168608</t>
-  </si>
-  <si>
-    <t>propuesta Nucleo rodete</t>
-  </si>
-  <si>
-    <t>benjamin.bustos@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>1213247778168609</t>
-  </si>
-  <si>
-    <t>propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>hugo isla martinez</t>
-  </si>
-  <si>
-    <t>hugo.isla@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC materiales</t>
-  </si>
-  <si>
-    <t>1213247778168610</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Alabe,Tableros OT 4214 ,rodete,Motor,Materiales a codigo // compras locales aprovisionamientomiento</t>
-  </si>
-  <si>
-    <t>1213247778168611</t>
-  </si>
-  <si>
-    <t>Alabe</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe,Fabricación Alabe</t>
-  </si>
-  <si>
-    <t>1213247781640415</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe,Alabe</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1213247781640416</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe</t>
-  </si>
-  <si>
-    <t>Alabe,Recepcion Alabe,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1213247781640417</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tableros OT 4214 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Tableros OT 4214 ,Fabricación Tablero OT 4214 </t>
-  </si>
-  <si>
-    <t>1213247781640418</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Tableros OT 4214 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Tablero OT 4214 ,Tableros OT 4214 </t>
-  </si>
-  <si>
-    <t>1213247781640419</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Tablero OT 4214 </t>
-  </si>
-  <si>
-    <t>Tableros OT 4214 ,RecepcionTableros,Recepcion Tableros</t>
-  </si>
-  <si>
-    <t>1213247781640420</t>
-  </si>
-  <si>
-    <t>rodete</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete,Fabricación  Rodete</t>
-  </si>
-  <si>
-    <t>1213247781640421</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>Fabricación  Rodete,rodete</t>
-  </si>
-  <si>
-    <t>1213247781640422</t>
-  </si>
-  <si>
-    <t>Fabricación  Rodete</t>
-  </si>
-  <si>
-    <t>rodete,Recepcion Rodete,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1213247781640423</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>Generación OC motor,Fabricaciónx motor,Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>1213247781640424</t>
-  </si>
-  <si>
-    <t>Generación OC motor</t>
-  </si>
-  <si>
-    <t>Fabricaciónx motor,Motor,Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>1213247781640425</t>
-  </si>
-  <si>
-    <t>Fabricaciónx motor</t>
-  </si>
-  <si>
-    <t>Motor,Recepcion Motor,Recepcion Motor</t>
-  </si>
-  <si>
-    <t>1213247781640426</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>Motor,Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213247781640427</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>1213247781640428</t>
-  </si>
-  <si>
-    <t>Generación OC materiales</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales,Materiales a codigo // compras locales aprovisionamientomiento</t>
-  </si>
-  <si>
-    <t>1213247781640429</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213575386156573</t>
-  </si>
-  <si>
-    <t>Ingenieria Y diseño</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos Definitivos,Check Planos,Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213575386156575</t>
-  </si>
-  <si>
-    <t>Planos Preliminar</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t>Planos Definitivos</t>
-  </si>
-  <si>
-    <t>1213575386156577</t>
-  </si>
-  <si>
-    <t>Planos Preliminar,Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>Check Planos,Ingenieria Y diseño</t>
-  </si>
-  <si>
-    <t>1213575386156579</t>
-  </si>
-  <si>
-    <t>Check Planos</t>
-  </si>
-  <si>
-    <t>Preparación de materiales,Armado,Montaje motor,Montaje Rodete,Montaje Alabe,Ingenieria Y diseño</t>
-  </si>
-  <si>
-    <t>1213575386156581</t>
-  </si>
-  <si>
-    <t>Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t>Pruebas FAT</t>
-  </si>
-  <si>
-    <t>Ingenieria Y diseño,RE-PINTADO</t>
-  </si>
-  <si>
-    <t>1213247781640432</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213247781640433</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
-  </si>
-  <si>
-    <t>1213247781640434</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>Bodega:,Preparación Materiales,Preparación de materiales</t>
-  </si>
-  <si>
-    <t>1213575386156541</t>
-  </si>
-  <si>
-    <t>Caldereria</t>
-  </si>
-  <si>
-    <t>Armado,Preparación de materiales,Control de calidad Aramado</t>
-  </si>
-  <si>
-    <t>1213575386156543</t>
-  </si>
-  <si>
-    <t>Preparación de materiales</t>
-  </si>
-  <si>
-    <t>Nicolás Mol</t>
-  </si>
-  <si>
-    <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Check Planos</t>
-  </si>
-  <si>
-    <t>1213575386156545</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Check Planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Aramado,Caldereria</t>
-  </si>
-  <si>
-    <t>1213575386156547</t>
-  </si>
-  <si>
-    <t>Control de calidad Aramado</t>
-  </si>
-  <si>
-    <t>Caldereria,Revestimiento</t>
-  </si>
-  <si>
-    <t>1213575386156613</t>
-  </si>
-  <si>
-    <t>bodega</t>
-  </si>
-  <si>
-    <t>Recepcion Motor,Recepcion Rodete,Recepcion Tableros,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1213575386156621</t>
-  </si>
-  <si>
-    <t>Recepcion Motor</t>
-  </si>
-  <si>
-    <t>bodega,Montaje motor</t>
-  </si>
-  <si>
-    <t>1213575386156619</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>bodega,Montaje Rodete</t>
-  </si>
-  <si>
-    <t>1213575386156617</t>
-  </si>
-  <si>
-    <t>bodega,Revision tableros pruebas</t>
-  </si>
-  <si>
-    <t>1213575386156615</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>bodega,Montaje Alabe</t>
-  </si>
-  <si>
-    <t>1213247781640444</t>
-  </si>
-  <si>
-    <t>Montaje:</t>
-  </si>
-  <si>
-    <t>Revestimiento,Montaje motor,Montaje Rodete,Montaje Alabe,Pruebas FAT,RE-PINTADO</t>
-  </si>
-  <si>
-    <t>1213247781640445</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>Montaje motor,Montaje Rodete,Montaje Alabe,Montaje:,Montaje motor</t>
-  </si>
-  <si>
-    <t>1213247781640446</t>
-  </si>
-  <si>
-    <t>Montaje motor</t>
-  </si>
-  <si>
-    <t>Revestimiento,Check Planos,Recepcion Motor</t>
-  </si>
-  <si>
-    <t>Pruebas FAT,Montaje:</t>
-  </si>
-  <si>
-    <t>1213247781640448</t>
-  </si>
-  <si>
-    <t>Montaje Rodete</t>
-  </si>
-  <si>
-    <t>Revestimiento,Check Planos,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1213247781640447</t>
-  </si>
-  <si>
-    <t>Montaje Alabe</t>
-  </si>
-  <si>
-    <t>Revestimiento,Check Planos,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1213247781640449</t>
-  </si>
-  <si>
-    <t>Montaje motor,Montaje Rodete,Montaje Alabe</t>
-  </si>
-  <si>
-    <t>Montaje:,Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213247781640450</t>
-  </si>
-  <si>
-    <t>RE-PINTADO</t>
-  </si>
-  <si>
-    <t>Montaje:,Coordinacion Entrega con Cliente</t>
-  </si>
-  <si>
-    <t>1213247781640451</t>
-  </si>
-  <si>
-    <t>Logistica:</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Embalaje,PACKING LIST,Despacho</t>
-  </si>
-  <si>
-    <t>1213247781640452</t>
-  </si>
-  <si>
-    <t>Karin Pinto</t>
-  </si>
-  <si>
-    <t>kpinto@zitron.com</t>
-  </si>
-  <si>
-    <t>RE-PINTADO,OT 4214 - TABLERO DE FUERZA SS ,Revision tableros pruebas</t>
-  </si>
-  <si>
-    <t>Logistica:,Embalaje</t>
-  </si>
-  <si>
-    <t>1213247781640453</t>
-  </si>
-  <si>
-    <t>Embalaje</t>
-  </si>
-  <si>
-    <t>PACKING LIST,Logistica:</t>
-  </si>
-  <si>
-    <t>1213247781640454</t>
-  </si>
-  <si>
-    <t>PACKING LIST</t>
-  </si>
-  <si>
-    <t>Despacho,Logistica:</t>
-  </si>
-  <si>
-    <t>1213247781640455</t>
-  </si>
-  <si>
-    <t>Despacho</t>
-  </si>
-  <si>
-    <t>Gestion,Costos,Logistica:,Instalación componentes</t>
-  </si>
-  <si>
-    <t>1213247781640456</t>
-  </si>
-  <si>
-    <t>Cierre proyecto:</t>
-  </si>
-  <si>
-    <t>Gestion,Costos</t>
-  </si>
-  <si>
-    <t>1213247781640457</t>
-  </si>
-  <si>
-    <t>Gestion</t>
-  </si>
-  <si>
-    <t>Nicolás</t>
-  </si>
-  <si>
-    <t>nicolas.tello@zitron.com</t>
   </si>
   <si>
     <t>1213247781640458</t>
@@ -1842,7 +1842,7 @@
         <v>46194.04721304398</v>
       </c>
       <c r="D10" s="5">
-        <v>46194.04723106482</v>
+        <v>46195.87486065972</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>45</v>
@@ -1876,13 +1876,9 @@
       </c>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
-      <c r="S10" s="6">
-        <v>1</v>
-      </c>
+      <c r="S10" s="6"/>
       <c r="T10" s="6"/>
-      <c r="U10" s="11" t="s">
-        <v>32</v>
-      </c>
+      <c r="U10" s="6"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
@@ -1960,7 +1956,7 @@
         <v>46191.89629966435</v>
       </c>
       <c r="D12" s="5">
-        <v>46191.89647877315</v>
+        <v>46195.87487971065</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>53</v>
@@ -2010,13 +2006,13 @@
       <c r="T12" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U12" s="12" t="s">
-        <v>58</v>
+      <c r="U12" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="8">
         <v>46127.62138719908</v>
@@ -2028,7 +2024,7 @@
         <v>46191.89628512731</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>26</v>
@@ -2061,7 +2057,7 @@
         <v>26</v>
       </c>
       <c r="P13" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
@@ -2071,7 +2067,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B14" s="5">
         <v>46065.78749844908</v>
@@ -2080,10 +2076,10 @@
         <v>46114.52385989584</v>
       </c>
       <c r="D14" s="5">
-        <v>46160.68150802083</v>
+        <v>46195.87482380787</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>25</v>
@@ -2107,24 +2103,20 @@
         <v>26</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P14" s="6" t="s">
         <v>26</v>
       </c>
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
-      <c r="S14" s="6">
-        <v>1</v>
-      </c>
+      <c r="S14" s="6"/>
       <c r="T14" s="6"/>
-      <c r="U14" s="11" t="s">
-        <v>32</v>
-      </c>
+      <c r="U14" s="6"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B15" s="8">
         <v>46065.78748841435</v>
@@ -2136,7 +2128,7 @@
         <v>46097.555050740746</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
@@ -2163,13 +2155,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q15" s="8">
         <v>46003</v>
@@ -2189,7 +2181,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" s="5">
         <v>46065.78749016204</v>
@@ -2201,7 +2193,7 @@
         <v>46114.52381064815</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2228,13 +2220,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q16" s="5">
         <v>46003</v>
@@ -2254,7 +2246,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17" s="8">
         <v>46065.78749607639</v>
@@ -2266,7 +2258,7 @@
         <v>46100.76562675926</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
@@ -2293,13 +2285,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O17" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="Q17" s="8">
         <v>46003</v>
@@ -2319,7 +2311,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B18" s="5">
         <v>46065.78749699074</v>
@@ -2331,7 +2323,7 @@
         <v>46114.52386047454</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
@@ -2358,13 +2350,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O18" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="Q18" s="5">
         <v>46003</v>
@@ -2384,7 +2376,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="8">
         <v>46065.78749806713</v>
@@ -2393,10 +2385,10 @@
         <v>46122.61313611111</v>
       </c>
       <c r="D19" s="8">
-        <v>46122.61315314815</v>
+        <v>46195.87478873842</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>25</v>
@@ -2420,24 +2412,20 @@
         <v>26</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
-      <c r="S19" s="9">
-        <v>1</v>
-      </c>
+      <c r="S19" s="9"/>
       <c r="T19" s="9"/>
-      <c r="U19" s="11" t="s">
-        <v>32</v>
-      </c>
+      <c r="U19" s="9"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B20" s="5">
         <v>46065.78749837963</v>
@@ -2449,7 +2437,7 @@
         <v>46097.55509811343</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2476,13 +2464,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Q20" s="5">
         <v>46007</v>
@@ -2502,7 +2490,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B21" s="8">
         <v>46065.78749869213</v>
@@ -2514,7 +2502,7 @@
         <v>46114.5239599537</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
@@ -2541,13 +2529,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q21" s="8">
         <v>46007</v>
@@ -2567,7 +2555,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B22" s="5">
         <v>46065.787499004626</v>
@@ -2579,7 +2567,7 @@
         <v>46097.55565678241</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
@@ -2606,13 +2594,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>48</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q22" s="5">
         <v>46007</v>
@@ -2632,7 +2620,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B23" s="8">
         <v>46065.78749934028</v>
@@ -2644,16 +2632,16 @@
         <v>46135.43274773148</v>
       </c>
       <c r="E23" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="F23" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>92</v>
-      </c>
       <c r="H23" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I23" s="8">
         <v>46007</v>
@@ -2671,13 +2659,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Q23" s="8">
         <v>46007</v>
@@ -2697,7 +2685,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B24" s="5">
         <v>46065.787488263886</v>
@@ -2709,16 +2697,16 @@
         <v>46100.790667037036</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G24" s="6" t="s">
+      <c r="H24" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I24" s="5">
         <v>46008</v>
@@ -2736,13 +2724,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q24" s="5">
         <v>46008</v>
@@ -2762,7 +2750,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B25" s="8">
         <v>46065.78748861111</v>
@@ -2771,10 +2759,10 @@
         <v>46191.89648689815</v>
       </c>
       <c r="D25" s="8">
-        <v>46195.87474907408</v>
+        <v>46195.87475449074</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>25</v>
@@ -2798,7 +2786,7 @@
         <v>26</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P25" s="9" t="s">
         <v>26</v>
@@ -2811,7 +2799,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B26" s="5">
         <v>46065.78748886574</v>
@@ -2823,16 +2811,16 @@
         <v>46118.8286340162</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G26" s="6" t="s">
+      <c r="H26" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I26" s="5">
         <v>46009</v>
@@ -2850,13 +2838,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q26" s="5">
         <v>46009</v>
@@ -2876,7 +2864,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27" s="8">
         <v>46065.78748912037</v>
@@ -2888,16 +2876,16 @@
         <v>46118.82821148148</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H27" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="I27" s="8">
         <v>46009</v>
@@ -2915,13 +2903,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
@@ -2929,15 +2917,15 @@
         <v>0</v>
       </c>
       <c r="T27" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U27" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U27" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B28" s="5">
         <v>46065.787489386574</v>
@@ -2949,16 +2937,16 @@
         <v>46118.82860748842</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I28" s="5">
         <v>46013</v>
@@ -2976,13 +2964,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -2990,15 +2978,15 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U28" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U28" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B29" s="8">
         <v>46065.7874896412</v>
@@ -3010,16 +2998,16 @@
         <v>46182.680279340275</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="I29" s="8">
         <v>46010</v>
@@ -3037,13 +3025,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q29" s="8">
         <v>46010</v>
@@ -3063,7 +3051,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="5">
         <v>46065.78748989583</v>
@@ -3075,16 +3063,16 @@
         <v>46169.84565782407</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I30" s="5">
         <v>46010</v>
@@ -3102,13 +3090,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3116,15 +3104,15 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U30" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U30" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B31" s="8">
         <v>46065.78749017361</v>
@@ -3136,16 +3124,16 @@
         <v>46182.68025478009</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="I31" s="8">
         <v>46106</v>
@@ -3163,13 +3151,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
@@ -3177,15 +3165,15 @@
         <v>0</v>
       </c>
       <c r="T31" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U31" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U31" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B32" s="5">
         <v>46065.78749045139</v>
@@ -3197,16 +3185,16 @@
         <v>46122.65076290509</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I32" s="5">
         <v>46009</v>
@@ -3224,13 +3212,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q32" s="5">
         <v>46009</v>
@@ -3250,7 +3238,7 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B33" s="8">
         <v>46065.787490717594</v>
@@ -3262,16 +3250,16 @@
         <v>46122.61608753473</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="I33" s="8">
         <v>46009</v>
@@ -3289,13 +3277,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
@@ -3303,15 +3291,15 @@
         <v>0</v>
       </c>
       <c r="T33" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U33" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U33" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B34" s="5">
         <v>46065.78748731481</v>
@@ -3323,16 +3311,16 @@
         <v>46122.61613047453</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I34" s="5">
         <v>46013</v>
@@ -3350,13 +3338,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -3364,15 +3352,15 @@
         <v>0</v>
       </c>
       <c r="T34" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U34" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U34" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B35" s="8">
         <v>46065.787487650465</v>
@@ -3384,16 +3372,16 @@
         <v>46097.55523409722</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="I35" s="8">
         <v>46009</v>
@@ -3411,13 +3399,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q35" s="8">
         <v>46009</v>
@@ -3437,7 +3425,7 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B36" s="5">
         <v>46065.78748796297</v>
@@ -3449,16 +3437,16 @@
         <v>46097.555153946756</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I36" s="5">
         <v>46009</v>
@@ -3476,13 +3464,13 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
@@ -3490,15 +3478,15 @@
         <v>0</v>
       </c>
       <c r="T36" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U36" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U36" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B37" s="8">
         <v>46065.78748824074</v>
@@ -3510,16 +3498,16 @@
         <v>46097.55519641204</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="I37" s="8">
         <v>46020</v>
@@ -3537,13 +3525,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
@@ -3551,15 +3539,15 @@
         <v>0</v>
       </c>
       <c r="T37" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U37" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U37" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B38" s="5">
         <v>46065.78748850695</v>
@@ -3571,16 +3559,16 @@
         <v>46097.55520825231</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="I38" s="5">
         <v>46020</v>
@@ -3598,13 +3586,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3612,15 +3600,15 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U38" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U38" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B39" s="8">
         <v>46065.787488773145</v>
@@ -3632,16 +3620,16 @@
         <v>46097.555442847224</v>
       </c>
       <c r="E39" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F39" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="9" t="s">
+      <c r="H39" s="9" t="s">
         <v>147</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>148</v>
       </c>
       <c r="I39" s="8">
         <v>46010</v>
@@ -3659,13 +3647,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q39" s="8">
         <v>46010</v>
@@ -3685,7 +3673,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B40" s="5">
         <v>46065.787489027774</v>
@@ -3697,16 +3685,16 @@
         <v>46097.55537814814</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="I40" s="5">
         <v>46010</v>
@@ -3724,13 +3712,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -3738,15 +3726,15 @@
         <v>0</v>
       </c>
       <c r="T40" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U40" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U40" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B41" s="8">
         <v>46065.78748929398</v>
@@ -3758,16 +3746,16 @@
         <v>46097.55541314815</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="H41" s="9" t="s">
         <v>147</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>148</v>
       </c>
       <c r="I41" s="8">
         <v>46021</v>
@@ -3785,13 +3773,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Q41" s="9"/>
       <c r="R41" s="9"/>
@@ -3799,15 +3787,15 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="U41" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="U41" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B42" s="5">
         <v>46090.78489178241</v>
@@ -3819,7 +3807,7 @@
         <v>46195.874716921295</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>25</v>
@@ -3843,7 +3831,7 @@
         <v>26</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -3856,7 +3844,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B43" s="8">
         <v>46090.78496228009</v>
@@ -3868,16 +3856,16 @@
         <v>46122.61600563658</v>
       </c>
       <c r="E43" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F43" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G43" s="9" t="s">
+      <c r="H43" s="9" t="s">
         <v>161</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>162</v>
       </c>
       <c r="I43" s="8">
         <v>46008</v>
@@ -3895,13 +3883,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q43" s="8">
         <v>46008</v>
@@ -3921,7 +3909,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B44" s="5">
         <v>46090.78503109954</v>
@@ -3933,16 +3921,16 @@
         <v>46122.616260069444</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="I44" s="5">
         <v>46029</v>
@@ -3960,13 +3948,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O44" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="P44" s="6" t="s">
         <v>165</v>
-      </c>
-      <c r="P44" s="6" t="s">
-        <v>166</v>
       </c>
       <c r="Q44" s="5">
         <v>46029</v>
@@ -3986,7 +3974,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B45" s="8">
         <v>46090.78508173611</v>
@@ -3998,16 +3986,16 @@
         <v>46122.61630149306</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="H45" s="9" t="s">
         <v>161</v>
-      </c>
-      <c r="H45" s="9" t="s">
-        <v>162</v>
       </c>
       <c r="I45" s="8">
         <v>46036</v>
@@ -4025,13 +4013,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Q45" s="8">
         <v>46036</v>
@@ -4051,7 +4039,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B46" s="5">
         <v>46090.78511145833</v>
@@ -4063,16 +4051,16 @@
         <v>46193.55680849537</v>
       </c>
       <c r="E46" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G46" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="F46" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G46" s="6" t="s">
+      <c r="H46" s="6" t="s">
         <v>172</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>173</v>
       </c>
       <c r="I46" s="6"/>
       <c r="J46" s="5">
@@ -4088,13 +4076,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O46" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="P46" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="P46" s="6" t="s">
-        <v>175</v>
       </c>
       <c r="Q46" s="5">
         <v>46071</v>
@@ -4114,7 +4102,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B47" s="8">
         <v>46065.78749037037</v>
@@ -4126,7 +4114,7 @@
         <v>46195.87468907407</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>25</v>
@@ -4150,7 +4138,7 @@
         <v>26</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="P47" s="9" t="s">
         <v>26</v>
@@ -4163,7 +4151,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B48" s="5">
         <v>46065.78749077546</v>
@@ -4175,16 +4163,16 @@
         <v>46122.61641002315</v>
       </c>
       <c r="E48" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G48" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G48" s="6" t="s">
+      <c r="H48" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="I48" s="5">
         <v>46041</v>
@@ -4202,13 +4190,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q48" s="5">
         <v>46041</v>
@@ -4228,7 +4216,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B49" s="8">
         <v>46065.7874911574</v>
@@ -4240,16 +4228,16 @@
         <v>46122.61645585648</v>
       </c>
       <c r="E49" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G49" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="F49" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G49" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>186</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>187</v>
       </c>
       <c r="I49" s="8">
         <v>46043</v>
@@ -4267,13 +4255,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Q49" s="8">
         <v>46043</v>
@@ -4293,7 +4281,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B50" s="5">
         <v>46090.77527482639</v>
@@ -4305,7 +4293,7 @@
         <v>46191.8965684838</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>25</v>
@@ -4329,7 +4317,7 @@
         <v>26</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4342,7 +4330,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B51" s="8">
         <v>46090.77537054398</v>
@@ -4354,16 +4342,16 @@
         <v>46122.61649803241</v>
       </c>
       <c r="E51" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G51" s="9" t="s">
+      <c r="H51" s="9" t="s">
         <v>194</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>195</v>
       </c>
       <c r="I51" s="8">
         <v>46045</v>
@@ -4381,13 +4369,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q51" s="8">
         <v>46045</v>
@@ -4407,7 +4395,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B52" s="5">
         <v>46090.775575486114</v>
@@ -4419,16 +4407,16 @@
         <v>46122.616699618055</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="H52" s="6" t="s">
         <v>194</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>195</v>
       </c>
       <c r="I52" s="5">
         <v>46050</v>
@@ -4446,13 +4434,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O52" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="P52" s="6" t="s">
         <v>199</v>
-      </c>
-      <c r="P52" s="6" t="s">
-        <v>200</v>
       </c>
       <c r="Q52" s="5">
         <v>46050</v>
@@ -4472,7 +4460,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B53" s="8">
         <v>46090.77562853009</v>
@@ -4484,16 +4472,16 @@
         <v>46122.61675327546</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="H53" s="9" t="s">
         <v>186</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>187</v>
       </c>
       <c r="I53" s="9"/>
       <c r="J53" s="8">
@@ -4509,13 +4497,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q53" s="8">
         <v>46057</v>
@@ -4535,7 +4523,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B54" s="5">
         <v>46090.792084768516</v>
@@ -4547,7 +4535,7 @@
         <v>46195.87467792824</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>25</v>
@@ -4571,7 +4559,7 @@
         <v>26</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P54" s="6" t="s">
         <v>26</v>
@@ -4584,7 +4572,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B55" s="8">
         <v>46090.79235962963</v>
@@ -4596,16 +4584,16 @@
         <v>46122.616780578704</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="H55" s="9" t="s">
         <v>181</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="I55" s="8">
         <v>46049</v>
@@ -4623,13 +4611,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P55" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q55" s="8">
         <v>46049</v>
@@ -4649,7 +4637,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B56" s="5">
         <v>46090.79230972222</v>
@@ -4661,16 +4649,16 @@
         <v>46122.61679635417</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="I56" s="5">
         <v>46031</v>
@@ -4688,13 +4676,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Q56" s="5">
         <v>46031</v>
@@ -4714,7 +4702,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B57" s="8">
         <v>46090.79220815972</v>
@@ -4732,10 +4720,10 @@
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="H57" s="9" t="s">
         <v>181</v>
-      </c>
-      <c r="H57" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="I57" s="9"/>
       <c r="J57" s="8">
@@ -4751,13 +4739,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="Q57" s="8">
         <v>46070</v>
@@ -4777,7 +4765,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B58" s="5">
         <v>46090.79211394676</v>
@@ -4789,16 +4777,16 @@
         <v>46122.61682444444</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="I58" s="5">
         <v>46015</v>
@@ -4816,13 +4804,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="Q58" s="5">
         <v>46015</v>
@@ -4842,7 +4830,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B59" s="8">
         <v>46065.787488692135</v>
@@ -4854,7 +4842,7 @@
         <v>46195.874617141206</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>25</v>
@@ -4878,7 +4866,7 @@
         <v>26</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>26</v>
@@ -4891,7 +4879,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B60" s="5">
         <v>46065.78748903935</v>
@@ -4903,16 +4891,16 @@
         <v>46127.61136859954</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I60" s="5">
         <v>46058</v>
@@ -4930,13 +4918,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Q60" s="5">
         <v>46058</v>
@@ -4956,7 +4944,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B61" s="8">
         <v>46065.787489560185</v>
@@ -4968,16 +4956,16 @@
         <v>46127.61151690972</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I61" s="8">
         <v>46065</v>
@@ -4995,13 +4983,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O61" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="P61" s="9" t="s">
         <v>226</v>
-      </c>
-      <c r="P61" s="9" t="s">
-        <v>227</v>
       </c>
       <c r="Q61" s="8">
         <v>46065</v>
@@ -5021,7 +5009,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B62" s="5">
         <v>46065.787495682875</v>
@@ -5033,16 +5021,16 @@
         <v>46127.61167162037</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I62" s="5">
         <v>46069</v>
@@ -5060,13 +5048,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Q62" s="5">
         <v>46069</v>
@@ -5086,7 +5074,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B63" s="8">
         <v>46065.78749190972</v>
@@ -5098,16 +5086,16 @@
         <v>46127.61154524305</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I63" s="8">
         <v>46066</v>
@@ -5125,13 +5113,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Q63" s="8">
         <v>46066</v>
@@ -5151,7 +5139,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B64" s="5">
         <v>46065.78749822917</v>
@@ -5163,16 +5151,16 @@
         <v>46191.78965548611</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I64" s="6"/>
       <c r="J64" s="5">
@@ -5188,13 +5176,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O64" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="P64" s="6" t="s">
         <v>235</v>
-      </c>
-      <c r="P64" s="6" t="s">
-        <v>236</v>
       </c>
       <c r="Q64" s="5">
         <v>46070</v>
@@ -5214,7 +5202,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B65" s="8">
         <v>46065.78749862268</v>
@@ -5226,16 +5214,16 @@
         <v>46195.87455763889</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I65" s="9"/>
       <c r="J65" s="8">
@@ -5251,13 +5239,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O65" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="Q65" s="8">
         <v>46072</v>
@@ -5275,7 +5263,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B66" s="5">
         <v>46065.78749923611</v>
@@ -5287,7 +5275,7 @@
         <v>46195.87453564815</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>25</v>
@@ -5311,7 +5299,7 @@
         <v>26</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>26</v>
@@ -5324,7 +5312,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B67" s="8">
         <v>46065.78748824074</v>
@@ -5336,16 +5324,16 @@
         <v>46195.868227858795</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="H67" s="9" t="s">
         <v>244</v>
-      </c>
-      <c r="H67" s="9" t="s">
-        <v>245</v>
       </c>
       <c r="I67" s="9"/>
       <c r="J67" s="8">
@@ -5361,13 +5349,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O67" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="P67" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="P67" s="9" t="s">
-        <v>247</v>
       </c>
       <c r="Q67" s="8">
         <v>46073</v>
@@ -5387,7 +5375,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B68" s="5">
         <v>46065.78748864583</v>
@@ -5399,16 +5387,16 @@
         <v>46195.87448907408</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I68" s="6"/>
       <c r="J68" s="5">
@@ -5424,13 +5412,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q68" s="5">
         <v>46078</v>
@@ -5450,7 +5438,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B69" s="8">
         <v>46065.787488946764</v>
@@ -5462,16 +5450,16 @@
         <v>46191.789935520836</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="H69" s="9" t="s">
         <v>194</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>195</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="8">
@@ -5487,13 +5475,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="P69" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="Q69" s="8">
         <v>46079</v>
@@ -5513,7 +5501,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B70" s="5">
         <v>46065.78748922454</v>
@@ -5525,16 +5513,16 @@
         <v>46191.79002724537</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>194</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>195</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5550,13 +5538,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Q70" s="5">
         <v>46080</v>
@@ -5576,7 +5564,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B71" s="8">
         <v>46065.78748953703</v>
@@ -5586,7 +5574,7 @@
         <v>46127.63253136574</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>25</v>
@@ -5610,7 +5598,7 @@
         <v>26</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="P71" s="9" t="s">
         <v>26</v>
@@ -5623,7 +5611,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B72" s="5">
         <v>46065.78748989583</v>
@@ -5633,16 +5621,16 @@
         <v>46191.79003109953</v>
       </c>
       <c r="E72" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G72" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="F72" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G72" s="6" t="s">
+      <c r="H72" s="6" t="s">
         <v>262</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>263</v>
       </c>
       <c r="I72" s="5">
         <v>46160</v>
@@ -5660,13 +5648,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q72" s="5">
         <v>46083</v>
@@ -5681,7 +5669,7 @@
         <v>31</v>
       </c>
       <c r="U72" s="12" t="s">
-        <v>58</v>
+        <v>263</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5702,10 +5690,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="H73" s="9" t="s">
         <v>262</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>263</v>
       </c>
       <c r="I73" s="8">
         <v>46160</v>
@@ -5723,13 +5711,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O73" s="9" t="s">
         <v>266</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q73" s="8">
         <v>46083</v>
@@ -5744,7 +5732,7 @@
         <v>31</v>
       </c>
       <c r="U73" s="12" t="s">
-        <v>58</v>
+        <v>263</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5836,7 +5824,7 @@
         <v>268</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P75" s="9" t="s">
         <v>272</v>
@@ -5854,7 +5842,7 @@
         <v>31</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>58</v>
+        <v>263</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -5917,7 +5905,7 @@
         <v>31</v>
       </c>
       <c r="U76" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>